<commit_message>
fix: repair garbled chinese in card config excels
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/BattleCardConfig.xlsx
+++ b/Design/Excel/ET/Datas/Game/BattleCardConfig.xlsx
@@ -530,8 +530,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ç©å®¶ææé-ç½®</t>
+          <t>玩家战斗配置</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -544,8 +543,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ç©å®¶é»è®¤å¡çææé-ç½®</t>
+          <t>玩家默认卡牌战斗配置</t>
         </is>
       </c>
     </row>

</xml_diff>